<commit_message>
Daily slate 2026-07-08 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-07-07.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-07-07.xlsx
@@ -503,13 +503,13 @@
         <v>11</v>
       </c>
       <c r="E3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" t="n">
         <v>5</v>
       </c>
-      <c r="F3" t="n">
-        <v>6</v>
-      </c>
       <c r="G3" t="n">
-        <v>45.5</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="4">
@@ -906,13 +906,13 @@
         <v>5342</v>
       </c>
       <c r="E17" t="n">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="F17" t="n">
-        <v>4351</v>
+        <v>4353</v>
       </c>
       <c r="G17" t="n">
-        <v>18.6</v>
+        <v>18.5</v>
       </c>
     </row>
   </sheetData>
@@ -1489,7 +1489,7 @@
         <v>170</v>
       </c>
       <c r="P7" t="n">
-        <v>18.6</v>
+        <v>18.5</v>
       </c>
       <c r="Q7" t="n">
         <v>5342</v>
@@ -1516,7 +1516,7 @@
         <v>130</v>
       </c>
       <c r="Z7" t="n">
-        <v>45.5</v>
+        <v>54.5</v>
       </c>
       <c r="AA7" t="n">
         <v>11</v>

</xml_diff>

<commit_message>
Daily slate 2026-07-09 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-07-07.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-07-07.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="E4" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="F4" t="n">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="G4" t="n">
-        <v>55</v>
+        <v>53.1</v>
       </c>
     </row>
     <row r="5">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="E7" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F7" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G7" t="n">
-        <v>46.9</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="8">
@@ -642,16 +642,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="E8" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F8" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="G8" t="n">
-        <v>50.8</v>
+        <v>50.4</v>
       </c>
     </row>
     <row r="9">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E9" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F9" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G9" t="n">
-        <v>66.7</v>
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="10">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="E10" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="F10" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G10" t="n">
-        <v>66.90000000000001</v>
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1055</v>
+        <v>1142</v>
       </c>
       <c r="E11" t="n">
-        <v>658</v>
+        <v>714</v>
       </c>
       <c r="F11" t="n">
-        <v>397</v>
+        <v>428</v>
       </c>
       <c r="G11" t="n">
-        <v>62.4</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>427</v>
+        <v>440</v>
       </c>
       <c r="E12" t="n">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="F12" t="n">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G12" t="n">
-        <v>44.7</v>
+        <v>46.1</v>
       </c>
     </row>
     <row r="13">
@@ -787,16 +787,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E13" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F13" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G13" t="n">
-        <v>58.6</v>
+        <v>56.5</v>
       </c>
     </row>
     <row r="14">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>348</v>
+        <v>375</v>
       </c>
       <c r="E14" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="F14" t="n">
-        <v>262</v>
+        <v>280</v>
       </c>
       <c r="G14" t="n">
-        <v>24.7</v>
+        <v>25.3</v>
       </c>
     </row>
     <row r="15">
@@ -845,13 +845,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>479</v>
+        <v>508</v>
       </c>
       <c r="E15" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F15" t="n">
-        <v>398</v>
+        <v>422</v>
       </c>
       <c r="G15" t="n">
         <v>16.9</v>
@@ -874,16 +874,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="E16" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F16" t="n">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="G16" t="n">
-        <v>9.4</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="17">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5342</v>
+        <v>5663</v>
       </c>
       <c r="E17" t="n">
-        <v>989</v>
+        <v>1069</v>
       </c>
       <c r="F17" t="n">
-        <v>4353</v>
+        <v>4594</v>
       </c>
       <c r="G17" t="n">
-        <v>18.5</v>
+        <v>18.9</v>
       </c>
     </row>
   </sheetData>
@@ -1158,10 +1158,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71.09999999999999</v>
+        <v>70.3</v>
       </c>
       <c r="C3" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D3" t="n">
         <v>73.5</v>
@@ -1215,10 +1215,10 @@
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>61.4</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="Y3" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="Z3" t="n">
         <v>100</v>
@@ -1236,10 +1236,10 @@
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>75</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="AG3" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55.2</v>
+        <v>50</v>
       </c>
       <c r="C4" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D4" t="n">
         <v>56.2</v>
@@ -1306,10 +1306,10 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>41.2</v>
+        <v>38.3</v>
       </c>
       <c r="Y4" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="Z4" t="n">
         <v>0</v>
@@ -1324,10 +1324,10 @@
         <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>62.5</v>
+        <v>63.2</v>
       </c>
       <c r="AG4" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -1447,52 +1447,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66.90000000000001</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="D7" t="n">
-        <v>62.4</v>
+        <v>62.5</v>
       </c>
       <c r="E7" t="n">
-        <v>1055</v>
+        <v>1142</v>
       </c>
       <c r="F7" t="n">
-        <v>44.7</v>
+        <v>46.1</v>
       </c>
       <c r="G7" t="n">
-        <v>427</v>
+        <v>440</v>
       </c>
       <c r="H7" t="n">
-        <v>58.6</v>
+        <v>56.5</v>
       </c>
       <c r="I7" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="J7" t="n">
-        <v>24.7</v>
+        <v>25.3</v>
       </c>
       <c r="K7" t="n">
-        <v>348</v>
+        <v>375</v>
       </c>
       <c r="L7" t="n">
         <v>16.9</v>
       </c>
       <c r="M7" t="n">
-        <v>479</v>
+        <v>508</v>
       </c>
       <c r="N7" t="n">
-        <v>9.4</v>
+        <v>10.1</v>
       </c>
       <c r="O7" t="n">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="P7" t="n">
-        <v>18.5</v>
+        <v>18.9</v>
       </c>
       <c r="Q7" t="n">
-        <v>5342</v>
+        <v>5663</v>
       </c>
       <c r="R7" t="n">
         <v>46.5</v>
@@ -1501,19 +1501,19 @@
         <v>43</v>
       </c>
       <c r="T7" t="n">
-        <v>55</v>
+        <v>53.1</v>
       </c>
       <c r="U7" t="n">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>50.8</v>
+        <v>50.4</v>
       </c>
       <c r="Y7" t="n">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="Z7" t="n">
         <v>54.5</v>
@@ -1528,16 +1528,16 @@
         <v>5</v>
       </c>
       <c r="AD7" t="n">
-        <v>46.9</v>
+        <v>45.8</v>
       </c>
       <c r="AE7" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="AF7" t="n">
-        <v>66.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="AG7" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>